<commit_message>
v1.3: one-click flow + single Excel for all classes
</commit_message>
<xml_diff>
--- a/sample_data/attendance_sample.xlsx
+++ b/sample_data/attendance_sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Attendance" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,208 +419,379 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>流水号</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>当前负责人</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Date Time</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Student</t>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Attendance</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Record Date</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>子表单</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2PI</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-08-03 09:00</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>HUI Ka Chun</t>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>子表单.Student</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>子表单.Name</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>子表单.Class</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2PI</t>
+          <t>已生效</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-08-03 09:00</t>
-        </is>
-      </c>
+          <t>202610150009</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LEUNG Charis,HUI Ting Him (Mack)</t>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Early Leave</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:37</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CHEUNG Sin Hang Enzo</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>CHEUNG Sin Hang Enzo</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4A</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2PI</t>
+          <t>已生效</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Casual Leave</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-08-04 09:00</t>
-        </is>
-      </c>
+          <t>202610150007</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>HUI Ka Chun</t>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:35</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CHEUNG Sin Hang Enzo,YAU Sze Wing Victoria,CHAN Chak Lam (Kalvin),CHU Lucas</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>CHEUNG Sin Hang Enzo,YAU Sze Wing Victoria,CHAN Chak Lam (Kalvin),CHU Lucas</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>4A,4A,4A,4A</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2PI</t>
+          <t>已生效</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Late</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-08-04 09:30</t>
-        </is>
-      </c>
+          <t>202610150006</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LEUNG Charis</t>
+          <t>4H(AM)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:35</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>KWUN Chak Him Hemera (Hemera),TSANG Lok Yan (Shanese),CHAM Nathaniel Lennon</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>KWUN Chak Him Hemera (Hemera),TSANG Lok Yan (Shanese),CHAM Nathaniel Lennon</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>4H(AM),4H(AM),4H(AM)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2PI</t>
+          <t>已生效</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sick Leave</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-08-05 09:00</t>
-        </is>
-      </c>
+          <t>202610150005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>HUI Ting Him (Mack)</t>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:34</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>CHEUNG Sin Hang Enzo,YAU Sze Wing Victoria,CHAN Chak Lam (Kalvin),CHU Lucas</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CHEUNG Sin Hang Enzo,YAU Sze Wing Victoria,CHAN Chak Lam (Kalvin),CHU Lucas</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>4A,4A,4A,4A</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2PI</t>
+          <t>已生效</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-08-05 09:00</t>
-        </is>
-      </c>
+          <t>202610160001</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>HUI Ka Chun,LEUNG Charis</t>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Sick Leave</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-10-16 09:00</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>YAU Sze Wing Victoria</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>YAU Sze Wing Victoria</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>4A</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2PI</t>
+          <t>已生效</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-08-06 09:00</t>
-        </is>
-      </c>
+          <t>202610160002</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>HUI Ka Chun,LEUNG Charis,HUI Ting Him (Mack)</t>
+          <t>4H(AM)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Casual Leave</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-10-16 09:00</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>TSANG Lok Yan (Shanese)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>TSANG Lok Yan (Shanese)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>4H(AM)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2P2</t>
+          <t>已生效</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-08-03 09:05</t>
-        </is>
-      </c>
+          <t>202610190001</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>WONG Siu Ming</t>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Late</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-10-19 09:45</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CHU Lucas</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>CHU Lucas</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>4A</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="G1:I1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>